<commit_message>
AP-08: schule.xlsx fuellen (Ferien und freie Tage)
Blatt "Ferien" mit 11 Eintraegen: Herbst-, Weihnachts-, Winter-, Oster-,
Pfingst- und Sommerferien, ein Brueckentag, zwei bewegliche Ferientage
(21.-22.12.2026, Leo 22.09.2026), Buss- und Bettag, Himmelfahrt,
Pfingstmontag. Jede Zeile mit Quelle (schulferien.eu bzw. kultus.sachsen.de,
beide laut Bericht noch nicht amtlich gegengeprueft).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/schule.xlsx
+++ b/content/schule.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="102">
   <si>
     <t>Hinweise zu schule.xlsx</t>
   </si>
@@ -221,6 +221,93 @@
   </si>
   <si>
     <t>zahnrad</t>
+  </si>
+  <si>
+    <t>schulferien.eu [nicht amtlich geprüft]</t>
+  </si>
+  <si>
+    <t>Weihnachtsferien</t>
+  </si>
+  <si>
+    <t>2026-12-23</t>
+  </si>
+  <si>
+    <t>2027-01-02</t>
+  </si>
+  <si>
+    <t>Winterferien</t>
+  </si>
+  <si>
+    <t>2027-02-08</t>
+  </si>
+  <si>
+    <t>2027-02-19</t>
+  </si>
+  <si>
+    <t>Osterferien</t>
+  </si>
+  <si>
+    <t>2027-03-26</t>
+  </si>
+  <si>
+    <t>2027-04-02</t>
+  </si>
+  <si>
+    <t>Pfingstferien</t>
+  </si>
+  <si>
+    <t>2027-05-15</t>
+  </si>
+  <si>
+    <t>2027-05-18</t>
+  </si>
+  <si>
+    <t>Sommerferien</t>
+  </si>
+  <si>
+    <t>2027-07-10</t>
+  </si>
+  <si>
+    <t>2027-08-20</t>
+  </si>
+  <si>
+    <t>Brückentag</t>
+  </si>
+  <si>
+    <t>2027-05-07</t>
+  </si>
+  <si>
+    <t>Bewegliche Ferientage</t>
+  </si>
+  <si>
+    <t>2026-12-21</t>
+  </si>
+  <si>
+    <t>2026-12-22</t>
+  </si>
+  <si>
+    <t>Leo 22.09.2026</t>
+  </si>
+  <si>
+    <t>Buß- und Bettag</t>
+  </si>
+  <si>
+    <t>2026-11-18</t>
+  </si>
+  <si>
+    <t>kultus.sachsen.de [zu prüfen]</t>
+  </si>
+  <si>
+    <t>Himmelfahrt</t>
+  </si>
+  <si>
+    <t>2027-05-06</t>
+  </si>
+  <si>
+    <t>Pfingstmontag</t>
+  </si>
+  <si>
+    <t>2027-05-17</t>
   </si>
   <si>
     <t>Stamm</t>
@@ -909,7 +996,7 @@
     <mergeCell ref="B17:D17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1069,13 +1156,13 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1097,10 +1184,164 @@
         <v>36</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1147,10 +1388,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>8</v>
@@ -1161,10 +1402,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>8</v>
@@ -1173,6 +1414,6 @@
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>